<commit_message>
Added timestamp reading and merging to one main csv
</commit_message>
<xml_diff>
--- a/Cubes_cHR_phosphorthermometry_27.05.26/Cube_natural_2cm_kHR_27.05.26.xlsx
+++ b/Cubes_cHR_phosphorthermometry_27.05.26/Cube_natural_2cm_kHR_27.05.26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\JedesAchteBild_27.05.26\converted_for_windows\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/izalewski/Documents/TU-Dortmund ISP Research/Cubes_cHR_phosphorthermometry_27.05.26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4995578B-99E8-4B5A-9348-42447A92B0A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6CA9475-561F-F24B-AC04-EF3147DE9EA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{15D49D2B-89F7-498E-A998-8CD5DA394A92}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17520" xr2:uid="{15D49D2B-89F7-498E-A998-8CD5DA394A92}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -102,16 +102,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -127,9 +125,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -167,7 +165,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -273,7 +271,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -415,7 +413,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -424,13 +422,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2891BD75-5A93-47B0-B5F3-B5A1D4C24EB5}">
   <dimension ref="A1:F306"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="33.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -450,7 +448,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>46169</v>
       </c>
@@ -470,227 +468,227 @@
         <v>704.99999999999989</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>46169</v>
       </c>
       <c r="B3" s="2">
         <v>0.41112268518518519</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="3">
         <v>0.4236111111111111</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="3">
         <v>1.2488425925925917E-2</v>
       </c>
       <c r="F3">
         <v>1078.9999999999991</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>46169</v>
       </c>
       <c r="B4" s="2">
         <v>0.41112268518518502</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4">
         <v>2</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="3">
         <v>0.42390046296296297</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="3">
         <v>1.2777777777777943E-2</v>
       </c>
       <c r="F4">
         <v>1104.0000000000143</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>46169</v>
       </c>
       <c r="B5" s="2">
         <v>0.41112268518518502</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5">
         <v>3</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="3">
         <v>0.42554398148148148</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="3">
         <v>1.442129629629646E-2</v>
       </c>
       <c r="F5">
         <v>1246.0000000000141</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>46169</v>
       </c>
       <c r="B6" s="2">
         <v>0.41112268518518502</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6">
         <v>4</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="3">
         <v>0.42773148148148149</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="3">
         <v>1.6608796296296469E-2</v>
       </c>
       <c r="F6">
         <v>1435.0000000000148</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>46169</v>
       </c>
       <c r="B7" s="2">
         <v>0.41112268518518502</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7">
         <v>5</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="3">
         <v>0.42885416666666665</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="3">
         <v>1.7731481481481626E-2</v>
       </c>
       <c r="F7">
         <v>1532.0000000000125</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>46169</v>
       </c>
       <c r="B8" s="2">
         <v>0.41112268518518502</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8">
         <v>6</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="3">
         <v>0.42917824074074074</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="3">
         <v>1.8055555555555713E-2</v>
       </c>
       <c r="F8">
         <v>1560.0000000000136</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>46169</v>
       </c>
       <c r="B9" s="2">
         <v>0.41112268518518502</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9">
         <v>7</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="3">
         <v>0.4302199074074074</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="3">
         <v>1.9097222222222376E-2</v>
       </c>
       <c r="F9">
         <v>1650.0000000000134</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>46169</v>
       </c>
       <c r="B10" s="2">
         <v>0.41112268518518502</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10">
         <v>8</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="3">
         <v>0.43078703703703702</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="3">
         <v>1.9664351851852002E-2</v>
       </c>
       <c r="F10">
         <v>1699.000000000013</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>46169</v>
       </c>
       <c r="B11" s="2">
         <v>0.41112268518518502</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11">
         <v>9</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="3">
         <v>0.43164351851851851</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="3">
         <v>2.0520833333333488E-2</v>
       </c>
       <c r="F11">
         <v>1773.0000000000134</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>46169</v>
       </c>
       <c r="B12" s="2">
         <v>0.41112268518518502</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12">
         <v>10</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="3">
         <v>0.43315972222222221</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="3">
         <v>2.2037037037037188E-2</v>
       </c>
       <c r="F12">
         <v>1904.000000000013</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>46169</v>
       </c>
       <c r="B13" s="2">
         <v>0.41112268518518502</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13">
         <v>11</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="3">
         <v>0.43334490740740739</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="3">
         <v>2.2222222222222365E-2</v>
       </c>
       <c r="F13">
         <v>1920.0000000000123</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>46169</v>
       </c>
@@ -710,7 +708,7 @@
         <v>2007.0000000000164</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>46169</v>
       </c>
@@ -730,7 +728,7 @@
         <v>2038.0000000000132</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>46169</v>
       </c>
@@ -750,7 +748,7 @@
         <v>2088.0000000000146</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>46169</v>
       </c>
@@ -770,7 +768,7 @@
         <v>2129.0000000000146</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>46169</v>
       </c>
@@ -790,7 +788,7 @@
         <v>2170.0000000000146</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>46169</v>
       </c>
@@ -810,7 +808,7 @@
         <v>2203.000000000015</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>46169</v>
       </c>
@@ -830,7 +828,7 @@
         <v>2233.000000000015</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>46169</v>
       </c>
@@ -850,7 +848,7 @@
         <v>2270.0000000000127</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>46169</v>
       </c>
@@ -870,7 +868,7 @@
         <v>2318.0000000000155</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>46169</v>
       </c>
@@ -890,7 +888,7 @@
         <v>2351.0000000000159</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>46169</v>
       </c>
@@ -910,7 +908,7 @@
         <v>2377.0000000000136</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>46169</v>
       </c>
@@ -930,7 +928,7 @@
         <v>2393.0000000000127</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>46169</v>
       </c>
@@ -950,7 +948,7 @@
         <v>2399.0000000000136</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>46169</v>
       </c>
@@ -970,7 +968,7 @@
         <v>2436.0000000000164</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>46169</v>
       </c>
@@ -990,7 +988,7 @@
         <v>2455.0000000000159</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>46169</v>
       </c>
@@ -1010,7 +1008,7 @@
         <v>2471.0000000000155</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>46169</v>
       </c>
@@ -1030,7 +1028,7 @@
         <v>2486.0000000000127</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>46169</v>
       </c>
@@ -1050,7 +1048,7 @@
         <v>2521.0000000000118</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>46169</v>
       </c>
@@ -1070,7 +1068,7 @@
         <v>2559.0000000000164</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>46169</v>
       </c>
@@ -1090,7 +1088,7 @@
         <v>2573.0000000000123</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>46169</v>
       </c>
@@ -1110,7 +1108,7 @@
         <v>2595.0000000000123</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>46169</v>
       </c>
@@ -1130,7 +1128,7 @@
         <v>2611.0000000000164</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>46169</v>
       </c>
@@ -1150,7 +1148,7 @@
         <v>2643.000000000015</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>46169</v>
       </c>
@@ -1170,7 +1168,7 @@
         <v>2660.0000000000159</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>46169</v>
       </c>
@@ -1190,7 +1188,7 @@
         <v>2677.0000000000123</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>46169</v>
       </c>
@@ -1210,7 +1208,7 @@
         <v>2699.0000000000127</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>46169</v>
       </c>
@@ -1230,7 +1228,7 @@
         <v>2729.0000000000127</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>46169</v>
       </c>
@@ -1250,7 +1248,7 @@
         <v>2748.0000000000123</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>46169</v>
       </c>
@@ -1270,7 +1268,7 @@
         <v>2766.000000000015</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>46169</v>
       </c>
@@ -1290,7 +1288,7 @@
         <v>2797.0000000000118</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>46169</v>
       </c>
@@ -1310,7 +1308,7 @@
         <v>2815.0000000000146</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>46169</v>
       </c>
@@ -1330,7 +1328,7 @@
         <v>2839.0000000000136</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>46169</v>
       </c>
@@ -1350,7 +1348,7 @@
         <v>2854.0000000000159</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>46169</v>
       </c>
@@ -1370,7 +1368,7 @@
         <v>2869.0000000000136</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>46169</v>
       </c>
@@ -1390,7 +1388,7 @@
         <v>2887.0000000000164</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>46169</v>
       </c>
@@ -1410,7 +1408,7 @@
         <v>2904.0000000000127</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>46169</v>
       </c>
@@ -1430,54 +1428,54 @@
         <v>2951.0000000000136</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="1"/>
       <c r="B51" s="2"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="1"/>
       <c r="B52" s="2"/>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="1"/>
       <c r="B53" s="2"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="1"/>
       <c r="B54" s="2"/>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="1"/>
       <c r="B55" s="2"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="1"/>
       <c r="B56" s="2"/>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="1"/>
       <c r="B57" s="2"/>
       <c r="D57" s="3"/>
       <c r="E57" s="3"/>
     </row>
-    <row r="75" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E75">
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E76">
         <v>0</v>
       </c>
@@ -1485,27 +1483,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E77">
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E78">
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E79">
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E80">
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E81">
         <v>0</v>
       </c>
@@ -1513,27 +1511,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E82">
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E83">
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E84">
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E85">
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E86">
         <v>0</v>
       </c>
@@ -1541,12 +1539,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E87">
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E148">
         <v>0</v>
       </c>
@@ -1554,27 +1552,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E149">
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E150">
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E151">
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E152">
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E153">
         <v>0</v>
       </c>
@@ -1582,27 +1580,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E154">
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E155">
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E156">
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E157">
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E158">
         <v>0</v>
       </c>
@@ -1610,17 +1608,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E159">
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E160">
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="251" spans="4:6" x14ac:dyDescent="0.2">
       <c r="D251" t="s">
         <v>0</v>
       </c>
@@ -1631,82 +1629,82 @@
         <v>2</v>
       </c>
     </row>
-    <row r="252" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="252" spans="4:6" x14ac:dyDescent="0.2">
       <c r="E252">
         <v>245</v>
       </c>
     </row>
-    <row r="253" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="253" spans="4:6" x14ac:dyDescent="0.2">
       <c r="E253">
         <v>250</v>
       </c>
     </row>
-    <row r="254" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="254" spans="4:6" x14ac:dyDescent="0.2">
       <c r="E254">
         <v>275</v>
       </c>
     </row>
-    <row r="255" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="255" spans="4:6" x14ac:dyDescent="0.2">
       <c r="E255">
         <v>300</v>
       </c>
     </row>
-    <row r="256" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="256" spans="4:6" x14ac:dyDescent="0.2">
       <c r="E256">
         <v>325</v>
       </c>
     </row>
-    <row r="257" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="257" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E257">
         <v>350</v>
       </c>
     </row>
-    <row r="258" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E258">
         <v>370</v>
       </c>
     </row>
-    <row r="259" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E259">
         <v>395</v>
       </c>
     </row>
-    <row r="260" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E260">
         <v>420</v>
       </c>
     </row>
-    <row r="261" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E261">
         <v>445</v>
       </c>
     </row>
-    <row r="262" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E262">
         <v>469</v>
       </c>
     </row>
-    <row r="263" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E263">
         <v>495</v>
       </c>
     </row>
-    <row r="264" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E264">
         <v>520</v>
       </c>
     </row>
-    <row r="265" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E265">
         <v>535</v>
       </c>
     </row>
-    <row r="266" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E266">
         <v>550</v>
       </c>
     </row>
-    <row r="276" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="276" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D276">
         <v>250</v>
       </c>
@@ -1714,7 +1712,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="277" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="277" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D277">
         <v>8.7237628341966004E-4</v>
       </c>
@@ -1722,7 +1720,7 @@
         <v>8.4999339550327895E-4</v>
       </c>
     </row>
-    <row r="278" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="278" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D278">
         <v>8.7629723680195202E-4</v>
       </c>
@@ -1730,7 +1728,7 @@
         <v>8.4927216129241701E-4</v>
       </c>
     </row>
-    <row r="279" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="279" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D279">
         <v>8.4902133303547001E-4</v>
       </c>
@@ -1738,7 +1736,7 @@
         <v>8.7728257215100697E-4</v>
       </c>
     </row>
-    <row r="280" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="280" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D280">
         <v>8.47350574208623E-4</v>
       </c>
@@ -1746,7 +1744,7 @@
         <v>8.56352922590513E-4</v>
       </c>
     </row>
-    <row r="281" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="281" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D281">
         <v>8.7010062018623804E-4</v>
       </c>
@@ -1754,7 +1752,7 @@
         <v>8.5971428973122797E-4</v>
       </c>
     </row>
-    <row r="282" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="282" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D282">
         <v>8.6523624504644897E-4</v>
       </c>
@@ -1762,7 +1760,7 @@
         <v>8.7298235789875795E-4</v>
       </c>
     </row>
-    <row r="283" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="283" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D283">
         <v>8.5037098461586999E-4</v>
       </c>
@@ -1770,7 +1768,7 @@
         <v>8.6721400935502299E-4</v>
       </c>
     </row>
-    <row r="284" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="284" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D284">
         <v>8.76149084672828E-4</v>
       </c>
@@ -1778,7 +1776,7 @@
         <v>8.6550612645823997E-4</v>
       </c>
     </row>
-    <row r="285" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="285" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D285">
         <v>8.4605674202877196E-4</v>
       </c>
@@ -1786,7 +1784,7 @@
         <v>8.4512686388397095E-4</v>
       </c>
     </row>
-    <row r="286" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="286" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D286">
         <v>8.5096561493668E-4</v>
       </c>
@@ -1794,7 +1792,7 @@
         <v>8.5742649447735999E-4</v>
       </c>
     </row>
-    <row r="287" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="287" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D287">
         <v>8.6039247189525418E-4</v>
       </c>
@@ -1802,7 +1800,7 @@
         <v>8.6008711933417952E-4</v>
       </c>
     </row>
-    <row r="288" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="288" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D288">
         <v>1.2069620116815019E-5</v>
       </c>
@@ -1810,7 +1808,7 @@
         <v>1.002969066327565E-5</v>
       </c>
     </row>
-    <row r="293" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="293" spans="4:6" x14ac:dyDescent="0.2">
       <c r="D293">
         <v>225</v>
       </c>
@@ -1821,7 +1819,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="304" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="304" spans="4:6" x14ac:dyDescent="0.2">
       <c r="D304" t="e">
         <v>#DIV/0!</v>
       </c>
@@ -1832,7 +1830,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="305" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="305" spans="4:6" x14ac:dyDescent="0.2">
       <c r="D305" t="e">
         <v>#DIV/0!</v>
       </c>
@@ -1843,7 +1841,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="306" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="306" spans="4:6" x14ac:dyDescent="0.2">
       <c r="D306" t="e">
         <v>#REF!</v>
       </c>

</xml_diff>